<commit_message>
fix: re-adiciona footer-bottom e implementa parametro Teto_Isencao
</commit_message>
<xml_diff>
--- a/out/calculadora-ir-configuracoes.xlsx
+++ b/out/calculadora-ir-configuracoes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30408"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Thais Camilo\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6A3ADE2B-3A2B-41D8-8BA0-528CDFCCB71D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A8DDD737-3A97-4953-9478-41F85FC87EDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Calculadora IRPF 2026" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>CALCULADORA IRPF 2026 (INCLUINDO ADICIONAL 10%)</t>
   </si>
@@ -116,6 +116,18 @@
   </si>
   <si>
     <t>Adicional_Aliquota</t>
+  </si>
+  <si>
+    <t>Ano_Base</t>
+  </si>
+  <si>
+    <t>Regra_Dividendos</t>
+  </si>
+  <si>
+    <t>PL 1087/26</t>
+  </si>
+  <si>
+    <t>Baseada no PL 1087/25 que prevê taxação de altas rendas.</t>
   </si>
 </sst>
 </file>
@@ -730,45 +742,65 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC854036-FFB5-45DC-AD7A-84466E74F51B}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>20</v>
       </c>
       <c r="B1" t="s">
         <v>21</v>
       </c>
-      <c r="E1" t="s">
+      <c r="D1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>23</v>
       </c>
       <c r="B2">
-        <v>189.59</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
+        <v>289.58999999999997</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
         <v>24</v>
       </c>
       <c r="B3">
-        <v>50000</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
       <c r="A4" t="s">
         <v>25</v>
       </c>
       <c r="B4">
         <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>